<commit_message>
Üst yönetime mail gönderimini ve görünürlüğünü tamamen engelle
Kapatma Onayı Bekleyen Kayıtlar ekranında üst yönetime ait cihaz kayıtları artık
listede hiç görünmüyor ve hiçbir yoldan (tekli/toplu/elle girilen alıcı) mail
gönderilemiyor. Kimlerin üst yönetim sayılacağı artık Excel'den okunmuyor — admin'in
Ayarlar > Veri Input'tan elle yönettiği sabit bir e-posta listesinden geliyor
(backend/src/routes/ustyonetim.js), TH'deki ünvan sütununa bağımlılık kaldırıldı.

Ayrıca demo verisindeki kalan gerçekçi olmayan kayıtlar düzeltildi: TH'deki
"Sentetik Cihaz (OBS)" placeholder satırları, TH'de eksik olan "Cihaz Sahibinin
Maili" sütunu, Kapatma Onayı/Yeni Kurulum'un asıl veri kaynağı olan yerel store'daki
eski "KULLANICI 117" tarzı sahte kayıtlar, SCCM/Lokasyon Mail Listesi'ndeki test
satırları ve eksik yerel lokasyon mailleri.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/demo-data/current/LokasyonMailListesi_20260921000000.xlsx
+++ b/backend/demo-data/current/LokasyonMailListesi_20260921000000.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E564"/>
+  <dimension ref="A1:E573"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9972,24 +9972,177 @@
     </row>
     <row r="564">
       <c r="A564" t="str">
-        <v>TESTA0</v>
+        <v>TR-SUBE-A</v>
       </c>
       <c r="B564" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="C564" t="str">
-        <v>suba-test@ornek.local</v>
+        <v>sube.a@thy.com</v>
       </c>
       <c r="D564" t="str">
         <v/>
       </c>
       <c r="E564" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="str">
+        <v>TR-SUBE-B</v>
+      </c>
+      <c r="B565" t="str">
+        <v>SUBE-B</v>
+      </c>
+      <c r="C565" t="str">
+        <v>sube.b@thy.com</v>
+      </c>
+      <c r="D565" t="str">
+        <v/>
+      </c>
+      <c r="E565" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="str">
+        <v>TR-SUBE-C</v>
+      </c>
+      <c r="B566" t="str">
+        <v>SUBE-C</v>
+      </c>
+      <c r="C566" t="str">
+        <v>sube.c@thy.com</v>
+      </c>
+      <c r="D566" t="str">
+        <v/>
+      </c>
+      <c r="E566" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="str">
+        <v>TR-MRKZ</v>
+      </c>
+      <c r="B567" t="str">
+        <v>MERKEZ BINA</v>
+      </c>
+      <c r="C567" t="str">
+        <v>merkezbina@thy.com</v>
+      </c>
+      <c r="D567" t="str">
+        <v/>
+      </c>
+      <c r="E567" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="str">
+        <v>TR-GNMD</v>
+      </c>
+      <c r="B568" t="str">
+        <v>GENEL MUDURLUK</v>
+      </c>
+      <c r="C568" t="str">
+        <v>genelmudurluk@thy.com</v>
+      </c>
+      <c r="D568" t="str">
+        <v/>
+      </c>
+      <c r="E568" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="str">
+        <v>TR-LOJM</v>
+      </c>
+      <c r="B569" t="str">
+        <v>LOJISTIK MERKEZI</v>
+      </c>
+      <c r="C569" t="str">
+        <v>lojistikmerkezi@thy.com</v>
+      </c>
+      <c r="D569" t="str">
+        <v/>
+      </c>
+      <c r="E569" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="str">
+        <v>TR-EGTM</v>
+      </c>
+      <c r="B570" t="str">
+        <v>EGITIM MERKEZI</v>
+      </c>
+      <c r="C570" t="str">
+        <v>egitimmerkezi@thy.com</v>
+      </c>
+      <c r="D570" t="str">
+        <v/>
+      </c>
+      <c r="E570" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="str">
+        <v>TR-SAHA1</v>
+      </c>
+      <c r="B571" t="str">
+        <v>SAHA OFISI-1</v>
+      </c>
+      <c r="C571" t="str">
+        <v>sahaofisi1@thy.com</v>
+      </c>
+      <c r="D571" t="str">
+        <v/>
+      </c>
+      <c r="E571" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="str">
+        <v>TR-SAHA2</v>
+      </c>
+      <c r="B572" t="str">
+        <v>SAHA OFISI-2</v>
+      </c>
+      <c r="C572" t="str">
+        <v>sahaofisi2@thy.com</v>
+      </c>
+      <c r="D572" t="str">
+        <v/>
+      </c>
+      <c r="E572" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="str">
+        <v>TR-DEPO1</v>
+      </c>
+      <c r="B573" t="str">
+        <v>DEPO-1</v>
+      </c>
+      <c r="C573" t="str">
+        <v>depo1@thy.com</v>
+      </c>
+      <c r="D573" t="str">
+        <v/>
+      </c>
+      <c r="E573" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E564"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E573"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>